<commit_message>
Save local changes before pulling
</commit_message>
<xml_diff>
--- a/pre-week-3/homework1_exercise1A.xlsx
+++ b/pre-week-3/homework1_exercise1A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eyerusalemdebero/Documents/DataAnalytics/pre-week-3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{857BF8F2-9D69-3242-ACE9-5ED50737AB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F096A03-6B28-D145-898A-19D2809903F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{423758B1-212B-F84F-A7BF-9DE776BCE4BB}"/>
+    <workbookView xWindow="2320" yWindow="740" windowWidth="11360" windowHeight="17220" xr2:uid="{423758B1-212B-F84F-A7BF-9DE776BCE4BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>